<commit_message>
new file:   ejercicioAmortizacion.xlsx deleted:    ejercicio_Amortizacion.xlsx new file:   ejerciciosAdicionales.ipynb new file:   enunciado.pdf modified:   modelos_python/IEPMBGPEII20262.ipynb deleted:    modelos_python/TrabajoFinal.ipynb new file:   plots/plot1_tc_chf_brl.png new file:   plots/plot2_capitalizacion.png modified:   pronosticos_uvr/pronostico_uvr_mbg.xlsx new file:   requirements.txt
</commit_message>
<xml_diff>
--- a/pronosticos_uvr/pronostico_uvr_mbg.xlsx
+++ b/pronosticos_uvr/pronostico_uvr_mbg.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H121"/>
+  <dimension ref="A1:H122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,10 +473,10 @@
         <v>378.080683427333</v>
       </c>
       <c r="D2" t="n">
-        <v>375.2260563401397</v>
+        <v>375.15296874899</v>
       </c>
       <c r="E2" t="n">
-        <v>381.0594930843304</v>
+        <v>380.9910983179209</v>
       </c>
       <c r="F2" t="n">
         <v>1.583583427333053</v>
@@ -499,10 +499,10 @@
         <v>379.8643420500457</v>
       </c>
       <c r="D3" t="n">
-        <v>375.8658607583487</v>
+        <v>375.7305953862398</v>
       </c>
       <c r="E3" t="n">
-        <v>383.9808588654782</v>
+        <v>383.9945694551324</v>
       </c>
       <c r="F3" t="n">
         <v>3.088042050045658</v>
@@ -525,10 +525,10 @@
         <v>381.6564153795173</v>
       </c>
       <c r="D4" t="n">
-        <v>376.5820935243045</v>
+        <v>376.6126106574155</v>
       </c>
       <c r="E4" t="n">
-        <v>386.740053824088</v>
+        <v>386.7087181793663</v>
       </c>
       <c r="F4" t="n">
         <v>3.493515379517362</v>
@@ -551,10 +551,10 @@
         <v>383.4569431135297</v>
       </c>
       <c r="D5" t="n">
-        <v>377.6610209680664</v>
+        <v>377.5271665858226</v>
       </c>
       <c r="E5" t="n">
-        <v>389.3033618208668</v>
+        <v>389.4470410207398</v>
       </c>
       <c r="F5" t="n">
         <v>2.803443113529681</v>
@@ -577,10 +577,10 @@
         <v>385.2659651371446</v>
       </c>
       <c r="D6" t="n">
-        <v>378.6603651888777</v>
+        <v>378.643773741209</v>
       </c>
       <c r="E6" t="n">
-        <v>392.0045294199632</v>
+        <v>391.8552614592119</v>
       </c>
       <c r="F6" t="n">
         <v>0.4549651371446544</v>
@@ -603,10 +603,10 @@
         <v>387.0835215235888</v>
       </c>
       <c r="D7" t="n">
-        <v>379.8070617007952</v>
+        <v>379.703067805694</v>
       </c>
       <c r="E7" t="n">
-        <v>394.4478745437053</v>
+        <v>394.3386573260057</v>
       </c>
       <c r="F7" t="n">
         <v>0.8486784764111803</v>
@@ -629,10 +629,10 @@
         <v>388.909652535141</v>
       </c>
       <c r="D8" t="n">
-        <v>381.0619939259742</v>
+        <v>380.9477471321787</v>
       </c>
       <c r="E8" t="n">
-        <v>396.911085250145</v>
+        <v>396.7604987216826</v>
       </c>
       <c r="F8" t="n">
         <v>1.352647464858933</v>
@@ -655,10 +655,10 @@
         <v>390.7443986240238</v>
       </c>
       <c r="D9" t="n">
-        <v>382.1477153479437</v>
+        <v>382.2332879361754</v>
       </c>
       <c r="E9" t="n">
-        <v>399.3327618540537</v>
+        <v>399.2169274838061</v>
       </c>
       <c r="F9" t="n">
         <v>1.388001375976216</v>
@@ -681,10 +681,10 @@
         <v>392.5878004333001</v>
       </c>
       <c r="D10" t="n">
-        <v>383.5787309447244</v>
+        <v>383.4518233590188</v>
       </c>
       <c r="E10" t="n">
-        <v>401.7819036734615</v>
+        <v>401.4782668934176</v>
       </c>
       <c r="F10" t="n">
         <v>0.3741995666998719</v>
@@ -707,10 +707,10 @@
         <v>394.4398987977731</v>
       </c>
       <c r="D11" t="n">
-        <v>384.8583505610551</v>
+        <v>384.8301238770864</v>
       </c>
       <c r="E11" t="n">
-        <v>404.0792668173071</v>
+        <v>403.9762530495971</v>
       </c>
       <c r="F11" t="n">
         <v>0.7199987977731439</v>
@@ -733,10 +733,10 @@
         <v>396.3007347448911</v>
       </c>
       <c r="D12" t="n">
-        <v>386.2858456469517</v>
+        <v>386.2367431992503</v>
       </c>
       <c r="E12" t="n">
-        <v>406.5968216684735</v>
+        <v>406.1705688457617</v>
       </c>
       <c r="F12" t="n">
         <v>1.673434744891154</v>
@@ -759,10 +759,10 @@
         <v>398.1703494956561</v>
       </c>
       <c r="D13" t="n">
-        <v>387.5658653506042</v>
+        <v>387.60364358824</v>
       </c>
       <c r="E13" t="n">
-        <v>409.0419569557821</v>
+        <v>408.5081501718503</v>
       </c>
       <c r="F13" t="n">
         <v>2.516449495656104</v>
@@ -785,10 +785,10 @@
         <v>400.048784465537</v>
       </c>
       <c r="D14" t="n">
-        <v>388.9532233943449</v>
+        <v>388.9159279078497</v>
       </c>
       <c r="E14" t="n">
-        <v>411.4224257007179</v>
+        <v>410.9987959652422</v>
       </c>
       <c r="F14" t="n">
         <v>3.42628446553698</v>
@@ -811,10 +811,10 @@
         <v>401.9360812653873</v>
       </c>
       <c r="D15" t="n">
-        <v>390.3333486435109</v>
+        <v>390.3764092109697</v>
       </c>
       <c r="E15" t="n">
-        <v>413.7574177687945</v>
+        <v>413.2426084465665</v>
       </c>
       <c r="F15" t="n">
         <v>4.813381265387306</v>
@@ -837,10 +837,10 @@
         <v>403.8322817023665</v>
       </c>
       <c r="D16" t="n">
-        <v>391.9183004151342</v>
+        <v>391.848544785404</v>
       </c>
       <c r="E16" t="n">
-        <v>416.0974253867355</v>
+        <v>415.7360058454459</v>
       </c>
       <c r="F16" t="n">
         <v>6.0218817023665</v>
@@ -863,10 +863,10 @@
         <v>405.7374277808663</v>
       </c>
       <c r="D17" t="n">
-        <v>393.2976856751687</v>
+        <v>393.2006433402432</v>
       </c>
       <c r="E17" t="n">
-        <v>418.4454000848809</v>
+        <v>418.1381563469798</v>
       </c>
       <c r="F17" t="n">
         <v>5.23222778086631</v>
@@ -889,10 +889,10 @@
         <v>407.6515617034412</v>
       </c>
       <c r="D18" t="n">
-        <v>394.7100799345231</v>
+        <v>394.7324663246154</v>
       </c>
       <c r="E18" t="n">
-        <v>420.5954721653728</v>
+        <v>420.3965145581824</v>
       </c>
       <c r="F18" t="n">
         <v>2.380761703441181</v>
@@ -915,10 +915,10 @@
         <v>409.5747258717432</v>
       </c>
       <c r="D19" t="n">
-        <v>396.2531898142115</v>
+        <v>396.1205010332379</v>
       </c>
       <c r="E19" t="n">
-        <v>423.0820168808885</v>
+        <v>422.7913672094382</v>
       </c>
       <c r="F19" t="n">
         <v>0.6062258717431632</v>
@@ -941,10 +941,10 @@
         <v>411.5069628874612</v>
       </c>
       <c r="D20" t="n">
-        <v>397.7489609018029</v>
+        <v>397.7785052325181</v>
       </c>
       <c r="E20" t="n">
-        <v>425.2807067211597</v>
+        <v>425.209878858775</v>
       </c>
       <c r="F20" t="n">
         <v>0.7031371125387977</v>
@@ -967,10 +967,10 @@
         <v>413.4483155532647</v>
       </c>
       <c r="D21" t="n">
-        <v>399.1961230822274</v>
+        <v>399.452689235068</v>
       </c>
       <c r="E21" t="n">
-        <v>427.6386362972717</v>
+        <v>427.8754867144764</v>
       </c>
       <c r="F21" t="n">
         <v>1.285684446735274</v>
@@ -993,10 +993,10 @@
         <v>415.3988268737519</v>
       </c>
       <c r="D22" t="n">
-        <v>400.9176472103313</v>
+        <v>400.7444250840875</v>
       </c>
       <c r="E22" t="n">
-        <v>429.9407401846987</v>
+        <v>430.2382419024276</v>
       </c>
       <c r="F22" t="n">
         <v>1.144673126248051</v>
@@ -1019,10 +1019,10 @@
         <v>417.3585400564024</v>
       </c>
       <c r="D23" t="n">
-        <v>402.3719435299796</v>
+        <v>402.5234653214933</v>
       </c>
       <c r="E23" t="n">
-        <v>432.4131470150766</v>
+        <v>432.5893642646765</v>
       </c>
       <c r="F23" t="n">
         <v>0.336259943597554</v>
@@ -1045,10 +1045,10 @@
         <v>419.3274985125342</v>
       </c>
       <c r="D24" t="n">
-        <v>403.8335024129543</v>
+        <v>404.0621323577355</v>
       </c>
       <c r="E24" t="n">
-        <v>434.8175889798925</v>
+        <v>434.9461173320141</v>
       </c>
       <c r="F24" t="n">
         <v>0.4747985125341643</v>
@@ -1071,10 +1071,10 @@
         <v>421.3057458582654</v>
       </c>
       <c r="D25" t="n">
-        <v>405.3596394922221</v>
+        <v>405.5041054908004</v>
       </c>
       <c r="E25" t="n">
-        <v>437.278613678171</v>
+        <v>437.4134879753642</v>
       </c>
       <c r="F25" t="n">
         <v>0.8364458582653924</v>
@@ -1095,10 +1095,10 @@
         <v>423.2933259154805</v>
       </c>
       <c r="D26" t="n">
-        <v>407.0133892361882</v>
+        <v>407.1546987042353</v>
       </c>
       <c r="E26" t="n">
-        <v>439.6638028584618</v>
+        <v>439.9826166993116</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
@@ -1113,10 +1113,10 @@
         <v>425.2902827128011</v>
       </c>
       <c r="D27" t="n">
-        <v>408.5234887649103</v>
+        <v>408.7822445882978</v>
       </c>
       <c r="E27" t="n">
-        <v>441.9282893028691</v>
+        <v>442.2331165674553</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
@@ -1131,10 +1131,10 @@
         <v>427.2966604865609</v>
       </c>
       <c r="D28" t="n">
-        <v>410.1806897830889</v>
+        <v>410.3666514265919</v>
       </c>
       <c r="E28" t="n">
-        <v>444.3038860784976</v>
+        <v>444.6952713739985</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
@@ -1149,10 +1149,10 @@
         <v>429.3125036817863</v>
       </c>
       <c r="D29" t="n">
-        <v>411.8118763199565</v>
+        <v>412.0796971120966</v>
       </c>
       <c r="E29" t="n">
-        <v>447.0857363391905</v>
+        <v>447.1226052638513</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
@@ -1167,10 +1167,10 @@
         <v>431.3378569531799</v>
       </c>
       <c r="D30" t="n">
-        <v>413.3212927784892</v>
+        <v>413.4689729539602</v>
       </c>
       <c r="E30" t="n">
-        <v>449.2235299251412</v>
+        <v>449.3753706540088</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
@@ -1185,10 +1185,10 @@
         <v>433.3727651661111</v>
       </c>
       <c r="D31" t="n">
-        <v>415.1456715662268</v>
+        <v>414.9897265680092</v>
       </c>
       <c r="E31" t="n">
-        <v>451.5411939387063</v>
+        <v>451.8580798185423</v>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
@@ -1203,10 +1203,10 @@
         <v>435.4172733976084</v>
       </c>
       <c r="D32" t="n">
-        <v>416.6591596346794</v>
+        <v>416.7955229235964</v>
       </c>
       <c r="E32" t="n">
-        <v>453.942943057551</v>
+        <v>454.3551335666094</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
@@ -1221,10 +1221,10 @@
         <v>437.4714269373591</v>
       </c>
       <c r="D33" t="n">
-        <v>418.275203681434</v>
+        <v>418.5188246885863</v>
       </c>
       <c r="E33" t="n">
-        <v>456.827023011459</v>
+        <v>456.880676006936</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
@@ -1239,10 +1239,10 @@
         <v>439.5352712887121</v>
       </c>
       <c r="D34" t="n">
-        <v>420.0726335917881</v>
+        <v>420.0973432347599</v>
       </c>
       <c r="E34" t="n">
-        <v>459.1032441621451</v>
+        <v>459.2050238629067</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
@@ -1257,10 +1257,10 @@
         <v>441.6088521696859</v>
       </c>
       <c r="D35" t="n">
-        <v>421.627829306235</v>
+        <v>421.7438189087717</v>
       </c>
       <c r="E35" t="n">
-        <v>461.5346585192425</v>
+        <v>461.6997066250599</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
@@ -1275,10 +1275,10 @@
         <v>443.6922155139812</v>
       </c>
       <c r="D36" t="n">
-        <v>423.4681957893018</v>
+        <v>423.3487547450005</v>
       </c>
       <c r="E36" t="n">
-        <v>464.0122272835332</v>
+        <v>464.1791672506281</v>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr"/>
@@ -1293,10 +1293,10 @@
         <v>445.785407471999</v>
       </c>
       <c r="D37" t="n">
-        <v>425.185589124448</v>
+        <v>425.0881283080262</v>
       </c>
       <c r="E37" t="n">
-        <v>466.7110462208126</v>
+        <v>466.6059096552993</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
@@ -1311,10 +1311,10 @@
         <v>447.888474411862</v>
       </c>
       <c r="D38" t="n">
-        <v>426.7578941876473</v>
+        <v>427.0766603204888</v>
       </c>
       <c r="E38" t="n">
-        <v>468.9454848321733</v>
+        <v>469.0668076461841</v>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
@@ -1329,10 +1329,10 @@
         <v>450.0014629204427</v>
       </c>
       <c r="D39" t="n">
-        <v>428.6584476411145</v>
+        <v>428.6151989312511</v>
       </c>
       <c r="E39" t="n">
-        <v>471.6208721124292</v>
+        <v>471.6175021873728</v>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
@@ -1347,10 +1347,10 @@
         <v>452.1244198043947</v>
       </c>
       <c r="D40" t="n">
-        <v>430.2754313082779</v>
+        <v>430.5618339483348</v>
       </c>
       <c r="E40" t="n">
-        <v>474.0585221140603</v>
+        <v>473.9860530237336</v>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
@@ -1365,10 +1365,10 @@
         <v>454.2573920911897</v>
       </c>
       <c r="D41" t="n">
-        <v>432.0319429431145</v>
+        <v>432.1573344208479</v>
       </c>
       <c r="E41" t="n">
-        <v>476.5426749683938</v>
+        <v>476.3962067898061</v>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
@@ -1383,10 +1383,10 @@
         <v>456.4004270301594</v>
       </c>
       <c r="D42" t="n">
-        <v>433.790661431504</v>
+        <v>434.0760742533831</v>
       </c>
       <c r="E42" t="n">
-        <v>478.8627100808625</v>
+        <v>478.9905493525557</v>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
@@ -1401,10 +1401,10 @@
         <v>458.5535720935424</v>
       </c>
       <c r="D43" t="n">
-        <v>435.5886123995808</v>
+        <v>435.866391767031</v>
       </c>
       <c r="E43" t="n">
-        <v>481.0671178376522</v>
+        <v>481.4298980670364</v>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
@@ -1419,10 +1419,10 @@
         <v>460.7168749775351</v>
       </c>
       <c r="D44" t="n">
-        <v>437.3230873015571</v>
+        <v>437.5874544181015</v>
       </c>
       <c r="E44" t="n">
-        <v>483.8472947440066</v>
+        <v>483.8224297428717</v>
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr"/>
@@ -1437,10 +1437,10 @@
         <v>462.8903836033489</v>
       </c>
       <c r="D45" t="n">
-        <v>439.3594929899684</v>
+        <v>439.2622735314858</v>
       </c>
       <c r="E45" t="n">
-        <v>486.100807521873</v>
+        <v>486.4699283264422</v>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
@@ -1455,10 +1455,10 @@
         <v>465.0741461182712</v>
       </c>
       <c r="D46" t="n">
-        <v>440.9840457780143</v>
+        <v>441.2725235428002</v>
       </c>
       <c r="E46" t="n">
-        <v>489.2521609476125</v>
+        <v>489.0091393378069</v>
       </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
@@ -1473,10 +1473,10 @@
         <v>467.2682108967326</v>
       </c>
       <c r="D47" t="n">
-        <v>442.8787190261417</v>
+        <v>443.1381321410056</v>
       </c>
       <c r="E47" t="n">
-        <v>491.6862626904804</v>
+        <v>491.59607997887</v>
       </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
@@ -1491,10 +1491,10 @@
         <v>469.472626541378</v>
       </c>
       <c r="D48" t="n">
-        <v>444.6833548889872</v>
+        <v>444.74635785813</v>
       </c>
       <c r="E48" t="n">
-        <v>494.4757083064065</v>
+        <v>494.1843560447089</v>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
@@ -1509,10 +1509,10 @@
         <v>471.6874418841433</v>
       </c>
       <c r="D49" t="n">
-        <v>446.2883940343661</v>
+        <v>446.6024871315167</v>
       </c>
       <c r="E49" t="n">
-        <v>496.7650517698067</v>
+        <v>497.0269262678191</v>
       </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr"/>
@@ -1527,10 +1527,10 @@
         <v>473.9127059873372</v>
       </c>
       <c r="D50" t="n">
-        <v>448.2130022672352</v>
+        <v>448.734384994414</v>
       </c>
       <c r="E50" t="n">
-        <v>499.6545979383263</v>
+        <v>499.7964773479019</v>
       </c>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr"/>
@@ -1545,10 +1545,10 @@
         <v>476.1484681447281</v>
       </c>
       <c r="D51" t="n">
-        <v>449.9816152376231</v>
+        <v>450.2858785714186</v>
       </c>
       <c r="E51" t="n">
-        <v>502.4524798385797</v>
+        <v>502.0925918292631</v>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
@@ -1563,10 +1563,10 @@
         <v>478.3947778826362</v>
       </c>
       <c r="D52" t="n">
-        <v>451.8173673490254</v>
+        <v>452.4817491496987</v>
       </c>
       <c r="E52" t="n">
-        <v>505.0773553518831</v>
+        <v>504.7395203096943</v>
       </c>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
@@ -1581,10 +1581,10 @@
         <v>480.6516849610297</v>
       </c>
       <c r="D53" t="n">
-        <v>453.4507715334765</v>
+        <v>454.0762315088605</v>
       </c>
       <c r="E53" t="n">
-        <v>507.8457089381511</v>
+        <v>507.4474074396958</v>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
@@ -1599,10 +1599,10 @@
         <v>482.9192393746283</v>
       </c>
       <c r="D54" t="n">
-        <v>455.4172508217621</v>
+        <v>455.8659356038081</v>
       </c>
       <c r="E54" t="n">
-        <v>510.3327083825407</v>
+        <v>510.244084438415</v>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
@@ -1617,10 +1617,10 @@
         <v>485.1974913540101</v>
       </c>
       <c r="D55" t="n">
-        <v>457.6699398759754</v>
+        <v>457.8734945998877</v>
       </c>
       <c r="E55" t="n">
-        <v>512.9255266020921</v>
+        <v>512.7214134555099</v>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr"/>
@@ -1635,10 +1635,10 @@
         <v>487.4864913667241</v>
       </c>
       <c r="D56" t="n">
-        <v>459.601778413262</v>
+        <v>459.8852000919351</v>
       </c>
       <c r="E56" t="n">
-        <v>514.9312882379122</v>
+        <v>515.5710952272042</v>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
@@ -1653,10 +1653,10 @@
         <v>489.7862901184084</v>
       </c>
       <c r="D57" t="n">
-        <v>461.4087726587384</v>
+        <v>461.8478762131899</v>
       </c>
       <c r="E57" t="n">
-        <v>517.9222683717195</v>
+        <v>517.9803561646213</v>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr"/>
@@ -1671,10 +1671,10 @@
         <v>492.0969385539136</v>
       </c>
       <c r="D58" t="n">
-        <v>463.4015750982739</v>
+        <v>464.0609383395472</v>
       </c>
       <c r="E58" t="n">
-        <v>520.5946205009941</v>
+        <v>520.9155861886793</v>
       </c>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr"/>
@@ -1689,10 +1689,10 @@
         <v>494.4184878584308</v>
       </c>
       <c r="D59" t="n">
-        <v>465.2367432090779</v>
+        <v>465.6874928398262</v>
       </c>
       <c r="E59" t="n">
-        <v>523.1490359628475</v>
+        <v>523.5482266034378</v>
       </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr"/>
@@ -1707,10 +1707,10 @@
         <v>496.7509894586261</v>
       </c>
       <c r="D60" t="n">
-        <v>467.3813085464789</v>
+        <v>467.4561415602061</v>
       </c>
       <c r="E60" t="n">
-        <v>525.857723061718</v>
+        <v>526.1343533270082</v>
       </c>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
@@ -1725,10 +1725,10 @@
         <v>499.0944950237793</v>
       </c>
       <c r="D61" t="n">
-        <v>469.526761034944</v>
+        <v>469.4763760528978</v>
       </c>
       <c r="E61" t="n">
-        <v>528.7631365289938</v>
+        <v>529.2291658958395</v>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
@@ -1743,10 +1743,10 @@
         <v>501.4490564669285</v>
       </c>
       <c r="D62" t="n">
-        <v>471.4462475901595</v>
+        <v>471.2897655936069</v>
       </c>
       <c r="E62" t="n">
-        <v>531.4964874282851</v>
+        <v>531.7174917721534</v>
       </c>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr"/>
@@ -1761,10 +1761,10 @@
         <v>503.8147259460206</v>
       </c>
       <c r="D63" t="n">
-        <v>473.5047398554226</v>
+        <v>473.4006227883683</v>
       </c>
       <c r="E63" t="n">
-        <v>534.2682751222367</v>
+        <v>534.7794230609607</v>
       </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
@@ -1779,10 +1779,10 @@
         <v>506.1915558650659</v>
       </c>
       <c r="D64" t="n">
-        <v>475.5195911368429</v>
+        <v>475.3632603418962</v>
       </c>
       <c r="E64" t="n">
-        <v>537.2636747807749</v>
+        <v>537.3814332351299</v>
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr"/>
@@ -1797,10 +1797,10 @@
         <v>508.5795988752996</v>
       </c>
       <c r="D65" t="n">
-        <v>477.7054378550015</v>
+        <v>477.3961346598401</v>
       </c>
       <c r="E65" t="n">
-        <v>539.6999596168432</v>
+        <v>540.3885777373528</v>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
@@ -1815,10 +1815,10 @@
         <v>510.9789078763476</v>
       </c>
       <c r="D66" t="n">
-        <v>479.8230910538568</v>
+        <v>479.4401897676243</v>
       </c>
       <c r="E66" t="n">
-        <v>543.0568726787118</v>
+        <v>543.252380062472</v>
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
@@ -1833,10 +1833,10 @@
         <v>513.3895360173991</v>
       </c>
       <c r="D67" t="n">
-        <v>481.3416057604654</v>
+        <v>481.3067060418632</v>
       </c>
       <c r="E67" t="n">
-        <v>545.8801931659955</v>
+        <v>546.1779689290915</v>
       </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr"/>
@@ -1851,10 +1851,10 @@
         <v>515.8115366983828</v>
       </c>
       <c r="D68" t="n">
-        <v>483.2449584906537</v>
+        <v>483.5062446875856</v>
       </c>
       <c r="E68" t="n">
-        <v>548.4823904893337</v>
+        <v>549.2820069828135</v>
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr"/>
@@ -1869,10 +1869,10 @@
         <v>518.2449635711511</v>
       </c>
       <c r="D69" t="n">
-        <v>485.504803652436</v>
+        <v>485.842263800086</v>
       </c>
       <c r="E69" t="n">
-        <v>551.5985013426935</v>
+        <v>551.7312356827804</v>
       </c>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr"/>
@@ -1887,10 +1887,10 @@
         <v>520.6898705406676</v>
       </c>
       <c r="D70" t="n">
-        <v>487.6961632035212</v>
+        <v>487.8437770899204</v>
       </c>
       <c r="E70" t="n">
-        <v>554.0283806195112</v>
+        <v>555.024996899361</v>
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
@@ -1905,10 +1905,10 @@
         <v>523.1463117662015</v>
       </c>
       <c r="D71" t="n">
-        <v>489.5531538722503</v>
+        <v>489.7063834825843</v>
       </c>
       <c r="E71" t="n">
-        <v>557.297553831075</v>
+        <v>557.5205660283225</v>
       </c>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr"/>
@@ -1923,10 +1923,10 @@
         <v>525.6143416625275</v>
       </c>
       <c r="D72" t="n">
-        <v>491.5603951584985</v>
+        <v>491.7251102689811</v>
       </c>
       <c r="E72" t="n">
-        <v>559.6012543115812</v>
+        <v>560.6173089346549</v>
       </c>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
@@ -1941,10 +1941,10 @@
         <v>528.0940149011312</v>
       </c>
       <c r="D73" t="n">
-        <v>493.3969931829009</v>
+        <v>494.0500852862392</v>
       </c>
       <c r="E73" t="n">
-        <v>562.4563522751982</v>
+        <v>563.402971770305</v>
       </c>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr"/>
@@ -1959,10 +1959,10 @@
         <v>530.5853864114198</v>
       </c>
       <c r="D74" t="n">
-        <v>495.3805021746913</v>
+        <v>495.7190080836083</v>
       </c>
       <c r="E74" t="n">
-        <v>565.5940532807776</v>
+        <v>566.3591909719898</v>
       </c>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr"/>
@@ -1977,10 +1977,10 @@
         <v>533.0885113819392</v>
       </c>
       <c r="D75" t="n">
-        <v>497.3643441604185</v>
+        <v>498.0843739423931</v>
       </c>
       <c r="E75" t="n">
-        <v>568.6416141972966</v>
+        <v>568.8594470569228</v>
       </c>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr"/>
@@ -1995,10 +1995,10 @@
         <v>535.6034452615966</v>
       </c>
       <c r="D76" t="n">
-        <v>499.4343336400773</v>
+        <v>500.5517157259337</v>
       </c>
       <c r="E76" t="n">
-        <v>571.6797399909535</v>
+        <v>571.6910606626057</v>
       </c>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
@@ -2013,10 +2013,10 @@
         <v>538.1302437608882</v>
       </c>
       <c r="D77" t="n">
-        <v>501.2374812052865</v>
+        <v>502.4449967148577</v>
       </c>
       <c r="E77" t="n">
-        <v>574.8860831577576</v>
+        <v>574.5772164759328</v>
       </c>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
@@ -2031,10 +2031,10 @@
         <v>540.6689628531346</v>
       </c>
       <c r="D78" t="n">
-        <v>503.3857339780993</v>
+        <v>504.5492601600729</v>
       </c>
       <c r="E78" t="n">
-        <v>578.0702423983428</v>
+        <v>577.5727723640762</v>
       </c>
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr"/>
@@ -2049,10 +2049,10 @@
         <v>543.2196587757192</v>
       </c>
       <c r="D79" t="n">
-        <v>505.6318569733879</v>
+        <v>506.7521540168064</v>
       </c>
       <c r="E79" t="n">
-        <v>581.0108622845523</v>
+        <v>580.6955263179348</v>
       </c>
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr"/>
@@ -2067,10 +2067,10 @@
         <v>545.7823880313344</v>
       </c>
       <c r="D80" t="n">
-        <v>508.0939172234038</v>
+        <v>509.0331709057556</v>
       </c>
       <c r="E80" t="n">
-        <v>584.3490010321448</v>
+        <v>583.8996148573269</v>
       </c>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr"/>
@@ -2085,10 +2085,10 @@
         <v>548.3572073892343</v>
       </c>
       <c r="D81" t="n">
-        <v>510.4923645554924</v>
+        <v>511.2395872803095</v>
       </c>
       <c r="E81" t="n">
-        <v>587.0128684374514</v>
+        <v>586.6859814659202</v>
       </c>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
@@ -2103,10 +2103,10 @@
         <v>550.9441738864909</v>
       </c>
       <c r="D82" t="n">
-        <v>512.4799083648875</v>
+        <v>513.4745900372753</v>
       </c>
       <c r="E82" t="n">
-        <v>589.5459741409704</v>
+        <v>589.4394892499788</v>
       </c>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
@@ -2121,10 +2121,10 @@
         <v>553.5433448292581</v>
       </c>
       <c r="D83" t="n">
-        <v>514.573105547629</v>
+        <v>515.6007596616066</v>
       </c>
       <c r="E83" t="n">
-        <v>592.4576779243059</v>
+        <v>592.8302001491866</v>
       </c>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr"/>
@@ -2139,10 +2139,10 @@
         <v>556.1547777940411</v>
       </c>
       <c r="D84" t="n">
-        <v>517.1815613985423</v>
+        <v>518.208037667575</v>
       </c>
       <c r="E84" t="n">
-        <v>595.612998305653</v>
+        <v>596.0064350715261</v>
       </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr"/>
@@ -2157,10 +2157,10 @@
         <v>558.7785306289721</v>
       </c>
       <c r="D85" t="n">
-        <v>519.5526745423246</v>
+        <v>520.40301496338</v>
       </c>
       <c r="E85" t="n">
-        <v>598.5144891841283</v>
+        <v>598.831524918542</v>
       </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr"/>
@@ -2175,10 +2175,10 @@
         <v>561.4146614550914</v>
       </c>
       <c r="D86" t="n">
-        <v>521.7617080081756</v>
+        <v>522.86278398631</v>
       </c>
       <c r="E86" t="n">
-        <v>602.0013372233088</v>
+        <v>601.8327931165629</v>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr"/>
@@ -2193,10 +2193,10 @@
         <v>564.0632286676347</v>
       </c>
       <c r="D87" t="n">
-        <v>524.000471821786</v>
+        <v>525.0370369659784</v>
       </c>
       <c r="E87" t="n">
-        <v>605.2852148293384</v>
+        <v>605.6926850579678</v>
       </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr"/>
@@ -2211,10 +2211,10 @@
         <v>566.7242909373275</v>
       </c>
       <c r="D88" t="n">
-        <v>526.0095517978773</v>
+        <v>527.5710308760669</v>
       </c>
       <c r="E88" t="n">
-        <v>608.5994036215495</v>
+        <v>609.1008199892121</v>
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr"/>
@@ -2229,10 +2229,10 @@
         <v>569.3979072116836</v>
       </c>
       <c r="D89" t="n">
-        <v>528.3415156111603</v>
+        <v>529.5765854460985</v>
       </c>
       <c r="E89" t="n">
-        <v>611.6109442754719</v>
+        <v>611.7839698027863</v>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
@@ -2247,10 +2247,10 @@
         <v>572.0841367163119</v>
       </c>
       <c r="D90" t="n">
-        <v>530.5169688701145</v>
+        <v>531.8192186886897</v>
       </c>
       <c r="E90" t="n">
-        <v>615.0282986452896</v>
+        <v>614.9929201699289</v>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr"/>
@@ -2265,10 +2265,10 @@
         <v>574.7830389562283</v>
       </c>
       <c r="D91" t="n">
-        <v>533.1849019343153</v>
+        <v>533.8747769954035</v>
       </c>
       <c r="E91" t="n">
-        <v>618.1432950985929</v>
+        <v>617.7995829554785</v>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr"/>
@@ -2283,10 +2283,10 @@
         <v>577.4946737171729</v>
       </c>
       <c r="D92" t="n">
-        <v>535.5528353587194</v>
+        <v>536.2638610430818</v>
       </c>
       <c r="E92" t="n">
-        <v>621.1642486061053</v>
+        <v>621.2219955069993</v>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
@@ -2301,10 +2301,10 @@
         <v>580.219101066935</v>
       </c>
       <c r="D93" t="n">
-        <v>537.7738326948729</v>
+        <v>538.8368341294204</v>
       </c>
       <c r="E93" t="n">
-        <v>624.2951094310154</v>
+        <v>624.6255453845869</v>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr"/>
@@ -2319,10 +2319,10 @@
         <v>582.9563813566842</v>
       </c>
       <c r="D94" t="n">
-        <v>540.3370507421803</v>
+        <v>540.8477986643104</v>
       </c>
       <c r="E94" t="n">
-        <v>627.5610018962177</v>
+        <v>627.109798247562</v>
       </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
@@ -2337,10 +2337,10 @@
         <v>585.7065752223065</v>
       </c>
       <c r="D95" t="n">
-        <v>542.3961264950476</v>
+        <v>542.9498144247664</v>
       </c>
       <c r="E95" t="n">
-        <v>630.6536328236737</v>
+        <v>630.503026173632</v>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
@@ -2355,10 +2355,10 @@
         <v>588.4697435857479</v>
       </c>
       <c r="D96" t="n">
-        <v>544.6856983826056</v>
+        <v>545.1970190381639</v>
       </c>
       <c r="E96" t="n">
-        <v>633.5837279877486</v>
+        <v>633.8680894084766</v>
       </c>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr"/>
@@ -2373,10 +2373,10 @@
         <v>591.2459476563637</v>
       </c>
       <c r="D97" t="n">
-        <v>546.7793871208562</v>
+        <v>547.569583044425</v>
       </c>
       <c r="E97" t="n">
-        <v>637.309385413856</v>
+        <v>637.0342025996595</v>
       </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr"/>
@@ -2391,10 +2391,10 @@
         <v>594.0352489322745</v>
       </c>
       <c r="D98" t="n">
-        <v>549.1599880391078</v>
+        <v>549.9868583264883</v>
       </c>
       <c r="E98" t="n">
-        <v>640.5815194847851</v>
+        <v>640.37545876994</v>
       </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr"/>
@@ -2409,10 +2409,10 @@
         <v>596.8377092017289</v>
       </c>
       <c r="D99" t="n">
-        <v>551.8690720383288</v>
+        <v>552.3643920424499</v>
       </c>
       <c r="E99" t="n">
-        <v>643.6076579078033</v>
+        <v>643.7202339587616</v>
       </c>
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr"/>
@@ -2427,10 +2427,10 @@
         <v>599.6533905444713</v>
       </c>
       <c r="D100" t="n">
-        <v>554.2634037229402</v>
+        <v>554.674299407242</v>
       </c>
       <c r="E100" t="n">
-        <v>646.870795059804</v>
+        <v>646.8553412982143</v>
       </c>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr"/>
@@ -2445,10 +2445,10 @@
         <v>602.4823553331182</v>
       </c>
       <c r="D101" t="n">
-        <v>556.8583092541551</v>
+        <v>557.2200073328149</v>
       </c>
       <c r="E101" t="n">
-        <v>649.9646063544178</v>
+        <v>650.0444613321038</v>
       </c>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr"/>
@@ -2463,10 +2463,10 @@
         <v>605.3246662345389</v>
       </c>
       <c r="D102" t="n">
-        <v>559.7006850817561</v>
+        <v>559.4114457361261</v>
       </c>
       <c r="E102" t="n">
-        <v>653.4865219812675</v>
+        <v>653.7975358684973</v>
       </c>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr"/>
@@ -2481,10 +2481,10 @@
         <v>608.1803862112441</v>
       </c>
       <c r="D103" t="n">
-        <v>562.3897902123131</v>
+        <v>561.9421450425053</v>
       </c>
       <c r="E103" t="n">
-        <v>656.5508885322211</v>
+        <v>657.2544604776376</v>
       </c>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr"/>
@@ -2499,10 +2499,10 @@
         <v>611.0495785227811</v>
       </c>
       <c r="D104" t="n">
-        <v>564.4521156110462</v>
+        <v>564.4776971647589</v>
       </c>
       <c r="E104" t="n">
-        <v>660.0028476246405</v>
+        <v>660.4086731922789</v>
       </c>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr"/>
@@ -2517,10 +2517,10 @@
         <v>613.932306727134</v>
       </c>
       <c r="D105" t="n">
-        <v>566.4783986671592</v>
+        <v>566.9101848090563</v>
       </c>
       <c r="E105" t="n">
-        <v>663.9043468950995</v>
+        <v>663.8790160622821</v>
       </c>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr"/>
@@ -2535,10 +2535,10 @@
         <v>616.8286346821329</v>
       </c>
       <c r="D106" t="n">
-        <v>568.8517047229782</v>
+        <v>569.2236997267485</v>
       </c>
       <c r="E106" t="n">
-        <v>667.362444940598</v>
+        <v>667.4843573251585</v>
       </c>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr"/>
@@ -2553,10 +2553,10 @@
         <v>619.7386265468674</v>
       </c>
       <c r="D107" t="n">
-        <v>571.0840111395491</v>
+        <v>571.2306696432514</v>
       </c>
       <c r="E107" t="n">
-        <v>670.3424138095228</v>
+        <v>670.7128610178229</v>
       </c>
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr"/>
@@ -2571,10 +2571,10 @@
         <v>622.6623467831085</v>
       </c>
       <c r="D108" t="n">
-        <v>573.7321398330701</v>
+        <v>573.7197351500542</v>
       </c>
       <c r="E108" t="n">
-        <v>673.9215756374556</v>
+        <v>674.1439992492562</v>
       </c>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr"/>
@@ -2589,10 +2589,10 @@
         <v>625.5998601567362</v>
       </c>
       <c r="D109" t="n">
-        <v>576.2754764910999</v>
+        <v>576.6337249150754</v>
       </c>
       <c r="E109" t="n">
-        <v>677.2071478652102</v>
+        <v>677.0893543755728</v>
       </c>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr"/>
@@ -2607,10 +2607,10 @@
         <v>628.5512317391746</v>
       </c>
       <c r="D110" t="n">
-        <v>578.5337894013845</v>
+        <v>579.4109120175256</v>
       </c>
       <c r="E110" t="n">
-        <v>680.6174611785889</v>
+        <v>680.3513442297717</v>
       </c>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr"/>
@@ -2625,10 +2625,10 @@
         <v>631.5165269088329</v>
       </c>
       <c r="D111" t="n">
-        <v>581.4768665940306</v>
+        <v>581.6251462359198</v>
       </c>
       <c r="E111" t="n">
-        <v>684.1186480477884</v>
+        <v>684.1382586419768</v>
       </c>
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr"/>
@@ -2643,10 +2643,10 @@
         <v>634.4958113525538</v>
       </c>
       <c r="D112" t="n">
-        <v>583.7705137643138</v>
+        <v>584.4158713730676</v>
       </c>
       <c r="E112" t="n">
-        <v>687.760887763942</v>
+        <v>687.6373102094662</v>
       </c>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr"/>
@@ -2661,10 +2661,10 @@
         <v>637.4891510670687</v>
       </c>
       <c r="D113" t="n">
-        <v>585.9623728626386</v>
+        <v>586.9282668732649</v>
       </c>
       <c r="E113" t="n">
-        <v>691.0131440761787</v>
+        <v>690.8519706969676</v>
       </c>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr"/>
@@ -2679,10 +2679,10 @@
         <v>640.4966123604595</v>
       </c>
       <c r="D114" t="n">
-        <v>588.7251825018132</v>
+        <v>589.4836966579943</v>
       </c>
       <c r="E114" t="n">
-        <v>694.5863344360184</v>
+        <v>694.2657732851155</v>
       </c>
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr"/>
@@ -2697,10 +2697,10 @@
         <v>643.5182618536279</v>
       </c>
       <c r="D115" t="n">
-        <v>590.8703909791045</v>
+        <v>592.102535816461</v>
       </c>
       <c r="E115" t="n">
-        <v>697.8661157536019</v>
+        <v>698.184660581489</v>
       </c>
       <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr"/>
@@ -2715,10 +2715,10 @@
         <v>646.55416648177</v>
       </c>
       <c r="D116" t="n">
-        <v>593.7387375439625</v>
+        <v>594.7011838230114</v>
       </c>
       <c r="E116" t="n">
-        <v>701.6755416680949</v>
+        <v>701.058289364436</v>
       </c>
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr"/>
@@ -2733,10 +2733,10 @@
         <v>649.6043934958608</v>
       </c>
       <c r="D117" t="n">
-        <v>596.175372933277</v>
+        <v>596.8012820046033</v>
       </c>
       <c r="E117" t="n">
-        <v>705.2632078062402</v>
+        <v>704.5859559789808</v>
       </c>
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr"/>
@@ -2751,10 +2751,10 @@
         <v>652.6690104641422</v>
       </c>
       <c r="D118" t="n">
-        <v>598.4754404023993</v>
+        <v>599.6649198030257</v>
       </c>
       <c r="E118" t="n">
-        <v>708.7061109296853</v>
+        <v>708.0443912740861</v>
       </c>
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr"/>
@@ -2769,10 +2769,10 @@
         <v>655.748085273621</v>
       </c>
       <c r="D119" t="n">
-        <v>600.9073595413226</v>
+        <v>602.2678045823541</v>
       </c>
       <c r="E119" t="n">
-        <v>712.7052787808158</v>
+        <v>711.3597753436087</v>
       </c>
       <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr"/>
@@ -2787,10 +2787,10 @@
         <v>658.841686131572</v>
       </c>
       <c r="D120" t="n">
-        <v>603.57926508129</v>
+        <v>604.5204281242617</v>
       </c>
       <c r="E120" t="n">
-        <v>715.9752102902614</v>
+        <v>715.1116041065565</v>
       </c>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr"/>
@@ -2805,14 +2805,32 @@
         <v>661.9498815670496</v>
       </c>
       <c r="D121" t="n">
-        <v>606.2939410775959</v>
+        <v>607.1219058676425</v>
       </c>
       <c r="E121" t="n">
-        <v>719.9187081149555</v>
+        <v>719.4998506218835</v>
       </c>
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="1" t="n">
+        <v>49278</v>
+      </c>
+      <c r="B122" t="inlineStr"/>
+      <c r="C122" t="n">
+        <v>665.0727404324048</v>
+      </c>
+      <c r="D122" t="n">
+        <v>610.1386345522751</v>
+      </c>
+      <c r="E122" t="n">
+        <v>723.1944433826457</v>
+      </c>
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="inlineStr"/>
+      <c r="H122" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>